<commit_message>
JAVA: [Eclipse] - Projekt "NMS_Viewer"   - neue Daten
git-svn-id: file:///G/_svn_repo/programming/JAVA-Projects%20-%20Eclipse/NMS_Viewer@4211 8592820e-bdd2-cc16-cb4b-ca06df7e8abd
</commit_message>
<xml_diff>
--- a/Konstruktion.xlsx
+++ b/Konstruktion.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\__Data\Eclipse - Workspace\NMS_Viewer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07192406-081A-4C76-865F-31E4C958692F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E6B22B-AEF1-438D-B56D-B459C5EA33CE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4EF5D9B1-307E-4186-869E-E042D9893C02}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -31,74 +32,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="43">
-  <si>
-    <t>^WALLLIGHTBLUE</t>
-  </si>
-  <si>
-    <t>0x00000000</t>
-  </si>
-  <si>
-    <t>( 0.5074 , -0.0004 , 0.8617 )</t>
-  </si>
-  <si>
-    <t>( 0.0003 , 1.0000 , 0.0003 )</t>
-  </si>
-  <si>
-    <t>Basiscomputer</t>
-  </si>
-  <si>
-    <t>^BASE_FLAG</t>
-  </si>
-  <si>
-    <t>( -0.01 , 0.02 , 0.00 )</t>
-  </si>
-  <si>
-    <t>( 0.0000 , -0.0000 , 1.0000 )</t>
-  </si>
-  <si>
-    <t>( 0.0000 , 1.0000 , -0.0000 )</t>
-  </si>
-  <si>
-    <t>Landefeld</t>
-  </si>
-  <si>
-    <t>^BUILDLANDINGPAD</t>
-  </si>
-  <si>
-    <t>( 17.83 , -0.19 , 16.58 )</t>
-  </si>
-  <si>
-    <t>Speicherpunkt</t>
-  </si>
-  <si>
-    <t>^BUILDSAVE</t>
-  </si>
-  <si>
-    <t>( -0.46 , -0.18 , 25.83 )</t>
-  </si>
-  <si>
-    <t>( 0.9787 , 0.0001 , -0.2051 )</t>
-  </si>
-  <si>
-    <t>( -0.0000 , 1.0000 , 0.0004 )</t>
-  </si>
-  <si>
-    <t>0x0000000B</t>
-  </si>
-  <si>
-    <t>^W_FLOOR</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>( 8.91 , -0.20 , 38.40 )</t>
   </si>
   <si>
-    <t>( -0.3797 , 0.0006 , -0.9251 )</t>
-  </si>
-  <si>
-    <t>( 0.0001 , 1.0000 , 0.0006 )</t>
-  </si>
-  <si>
     <t>( 3.97 , -0.20 , 40.42 )</t>
   </si>
   <si>
@@ -108,58 +46,88 @@
     <t>( 6.88 , -0.20 , 33.46 )</t>
   </si>
   <si>
-    <t>^W_DOOR</t>
-  </si>
-  <si>
-    <t>( 9.92 , -0.20 , 40.86 )</t>
-  </si>
-  <si>
-    <t>( 11.38 , -0.20 , 37.38 )</t>
-  </si>
-  <si>
-    <t>( -0.9251 , -0.0001 , 0.3797 )</t>
-  </si>
-  <si>
     <t>( 8.91 , 3.13 , 38.40 )</t>
   </si>
   <si>
-    <t>( 6.44 , -0.20 , 39.41 )</t>
-  </si>
-  <si>
-    <t>( 0.9251 , 0.0001 , -0.3797 )</t>
-  </si>
-  <si>
     <t>( 5.36 , 2.19 , 37.18 )</t>
   </si>
   <si>
-    <t>( -0.0001 , -1.0000 , -0.0006 )</t>
-  </si>
-  <si>
     <t>( 5.65 , 2.19 , 37.09 )</t>
   </si>
   <si>
-    <t>^W_WALL</t>
-  </si>
-  <si>
-    <t>( 4.99 , -0.20 , 42.89 )</t>
-  </si>
-  <si>
-    <t>^W_GFLOOR</t>
-  </si>
-  <si>
-    <t>( 3.98 , 3.13 , 40.42 )</t>
-  </si>
-  <si>
-    <t>^W_DOORWINDOW</t>
-  </si>
-  <si>
-    <t>( 1.51 , -0.20 , 41.43 )</t>
-  </si>
-  <si>
-    <t>^W_WALL_WINDOW</t>
-  </si>
-  <si>
-    <t>( -0.52 , -0.20 , 36.50 )</t>
+    <t>^M_ARCH</t>
+  </si>
+  <si>
+    <t>^M_ARCH_H</t>
+  </si>
+  <si>
+    <t>^M_DOOR</t>
+  </si>
+  <si>
+    <t>^M_DOORWINDOW</t>
+  </si>
+  <si>
+    <t>^M_DOOR_H</t>
+  </si>
+  <si>
+    <t>^M_FLOOR</t>
+  </si>
+  <si>
+    <t>^M_FLOOR_Q</t>
+  </si>
+  <si>
+    <t>^M_GDOOR</t>
+  </si>
+  <si>
+    <t>^M_GDOOR_D</t>
+  </si>
+  <si>
+    <t>^M_GFLOOR</t>
+  </si>
+  <si>
+    <t>^M_RAMP</t>
+  </si>
+  <si>
+    <t>^M_RAMP_H</t>
+  </si>
+  <si>
+    <t>^M_ROOF</t>
+  </si>
+  <si>
+    <t>^M_ROOF_C</t>
+  </si>
+  <si>
+    <t>^M_ROOF_IC</t>
+  </si>
+  <si>
+    <t>^M_ROOF_M</t>
+  </si>
+  <si>
+    <t>^M_SDOOR</t>
+  </si>
+  <si>
+    <t>^M_TRIFLOOR</t>
+  </si>
+  <si>
+    <t>^M_TRIFLOOR_Q</t>
+  </si>
+  <si>
+    <t>^M_WALL</t>
+  </si>
+  <si>
+    <t>^M_WALLDIAGONAL</t>
+  </si>
+  <si>
+    <t>^M_WALL_H</t>
+  </si>
+  <si>
+    <t>^M_WALL_Q</t>
+  </si>
+  <si>
+    <t>^M_WALL_Q_H</t>
+  </si>
+  <si>
+    <t>^M_WALL_WINDOW</t>
   </si>
 </sst>
 </file>
@@ -524,16 +492,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5801AF08-4A3E-4CFE-B210-4C3C7BEC84B7}">
-  <dimension ref="B4:U26"/>
+  <dimension ref="B4:U28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" customWidth="1"/>
+    <col min="7" max="7" width="29.7109375" customWidth="1"/>
+    <col min="8" max="8" width="26.28515625" customWidth="1"/>
     <col min="9" max="9" width="4.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="4.42578125" customWidth="1"/>
     <col min="11" max="11" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -544,194 +512,110 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B4" s="2">
-        <v>43801.434432870374</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>8</v>
-      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B5" s="2">
-        <v>43801.440578703703</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>3</v>
-      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B6" s="2">
-        <v>43801.570590277777</v>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="2:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="B7" s="2">
-        <v>43801.577824074076</v>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="2:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
-        <v>43801.577824074076</v>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B9" s="2">
-        <v>43801.562905092593</v>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B10" s="2">
-        <v>43801.562928240739</v>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B11" s="2">
-        <v>43801.562951388885</v>
+      <c r="B11" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="L11">
         <f>FIND(" , ",K11)</f>
@@ -771,29 +655,19 @@
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B12" s="2">
-        <v>43801.562962962962</v>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="L12">
         <f>FIND(" , ",K12)</f>
@@ -833,25 +707,15 @@
       </c>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B13" s="2">
-        <v>43801.563078703701</v>
+      <c r="B13" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="R13">
@@ -872,52 +736,32 @@
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B14" s="2">
-        <v>43801.563101851854</v>
+      <c r="B14" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B15" s="2">
-        <v>43801.56318287037</v>
+      <c r="B15" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="L15">
         <f>FIND(" , ",K15)</f>
@@ -957,29 +801,19 @@
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B16" s="2">
-        <v>43801.577326388891</v>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
       <c r="K16" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="L16">
         <f>FIND(" , ",K16)</f>
@@ -1019,25 +853,15 @@
       </c>
     </row>
     <row r="17" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B17" s="2">
-        <v>43801.577453703707</v>
+      <c r="B17" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="C17" s="3"/>
-      <c r="D17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="R17">
@@ -1058,52 +882,32 @@
       </c>
     </row>
     <row r="18" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B18" s="2">
-        <v>43801.577824074076</v>
+      <c r="B18" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="C18" s="3"/>
-      <c r="D18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="2:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="2">
-        <v>43801.577615740738</v>
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="C19" s="3"/>
-      <c r="D19" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="L19">
         <f>FIND(" , ",K19)</f>
@@ -1143,31 +947,19 @@
       </c>
     </row>
     <row r="20" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B20" s="2">
-        <v>43801.44363425926</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="B20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="L20">
         <f>FIND(" , ",K20)</f>
@@ -1207,6 +999,9 @@
       </c>
     </row>
     <row r="21" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
       <c r="R21">
         <f>R19-R20</f>
         <v>0</v>
@@ -1224,9 +1019,22 @@
         <v>3.33</v>
       </c>
     </row>
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+    </row>
     <row r="24" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
       <c r="K24" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="L24">
         <f>FIND(" , ",K24)</f>
@@ -1266,8 +1074,11 @@
       </c>
     </row>
     <row r="25" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
       <c r="K25" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="L25">
         <f>FIND(" , ",K25)</f>
@@ -1307,6 +1118,9 @@
       </c>
     </row>
     <row r="26" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
       <c r="R26">
         <f>R24-R25</f>
         <v>-0.29000000000000004</v>
@@ -1324,7 +1138,26 @@
         <v>0.30364452901377847</v>
       </c>
     </row>
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86F96532-323F-4EE8-9F49-D2C9B7BC1DE1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>